<commit_message>
Dela upp ACL-motorlager i Vevlager/Ramlager/Axiallager
</commit_message>
<xml_diff>
--- a/ny-hemsida/produkter.xlsx
+++ b/ny-hemsida/produkter.xlsx
@@ -15225,7 +15225,7 @@
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
@@ -15263,7 +15263,7 @@
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B391" t="inlineStr">
@@ -15301,7 +15301,7 @@
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Axiallager</t>
         </is>
       </c>
       <c r="B392" t="inlineStr">
@@ -15339,7 +15339,7 @@
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B393" t="inlineStr">
@@ -15377,7 +15377,7 @@
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B394" t="inlineStr">
@@ -15415,7 +15415,7 @@
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
@@ -15453,7 +15453,7 @@
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
@@ -15491,7 +15491,7 @@
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B397" t="inlineStr">
@@ -15529,7 +15529,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B398" t="inlineStr">
@@ -15567,7 +15567,7 @@
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B399" t="inlineStr">
@@ -15605,7 +15605,7 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Axiallager</t>
         </is>
       </c>
       <c r="B400" t="inlineStr">
@@ -15643,7 +15643,7 @@
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B401" t="inlineStr">
@@ -15681,7 +15681,7 @@
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B402" t="inlineStr">
@@ -15719,7 +15719,7 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B403" t="inlineStr">
@@ -15757,7 +15757,7 @@
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B404" t="inlineStr">
@@ -15795,7 +15795,7 @@
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B405" t="inlineStr">
@@ -15833,7 +15833,7 @@
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Axiallager</t>
         </is>
       </c>
       <c r="B406" t="inlineStr">
@@ -15871,7 +15871,7 @@
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B407" t="inlineStr">
@@ -15909,7 +15909,7 @@
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B408" t="inlineStr">
@@ -15947,7 +15947,7 @@
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B409" t="inlineStr">
@@ -15985,7 +15985,7 @@
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B410" t="inlineStr">
@@ -16023,7 +16023,7 @@
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B411" t="inlineStr">
@@ -16061,7 +16061,7 @@
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B412" t="inlineStr">
@@ -16099,7 +16099,7 @@
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B413" t="inlineStr">
@@ -16137,7 +16137,7 @@
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B414" t="inlineStr">
@@ -16175,7 +16175,7 @@
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B415" t="inlineStr">
@@ -16213,7 +16213,7 @@
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B416" t="inlineStr">
@@ -16251,7 +16251,7 @@
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B417" t="inlineStr">
@@ -16289,7 +16289,7 @@
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B418" t="inlineStr">
@@ -16327,7 +16327,7 @@
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B419" t="inlineStr">
@@ -16365,7 +16365,7 @@
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B420" t="inlineStr">
@@ -16403,7 +16403,7 @@
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B421" t="inlineStr">
@@ -16441,7 +16441,7 @@
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B422" t="inlineStr">
@@ -16479,7 +16479,7 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B423" t="inlineStr">
@@ -16517,7 +16517,7 @@
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B424" t="inlineStr">
@@ -16555,7 +16555,7 @@
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B425" t="inlineStr">
@@ -16593,7 +16593,7 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B426" t="inlineStr">
@@ -16631,7 +16631,7 @@
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B427" t="inlineStr">
@@ -16707,7 +16707,7 @@
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B429" t="inlineStr">
@@ -16745,7 +16745,7 @@
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B430" t="inlineStr">
@@ -16783,7 +16783,7 @@
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B431" t="inlineStr">
@@ -16821,7 +16821,7 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B432" t="inlineStr">
@@ -16859,7 +16859,7 @@
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B433" t="inlineStr">
@@ -16897,7 +16897,7 @@
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B434" t="inlineStr">
@@ -16935,7 +16935,7 @@
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B435" t="inlineStr">
@@ -16973,7 +16973,7 @@
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B436" t="inlineStr">
@@ -17011,7 +17011,7 @@
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B437" t="inlineStr">
@@ -17049,7 +17049,7 @@
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B438" t="inlineStr">
@@ -17087,7 +17087,7 @@
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B439" t="inlineStr">
@@ -17125,7 +17125,7 @@
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B440" t="inlineStr">
@@ -17163,7 +17163,7 @@
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B441" t="inlineStr">
@@ -17201,7 +17201,7 @@
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
@@ -17239,7 +17239,7 @@
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
@@ -17277,7 +17277,7 @@
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
@@ -17315,7 +17315,7 @@
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
@@ -17353,7 +17353,7 @@
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B446" t="inlineStr">
@@ -17391,7 +17391,7 @@
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B447" t="inlineStr">
@@ -17429,7 +17429,7 @@
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B448" t="inlineStr">
@@ -17467,7 +17467,7 @@
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B449" t="inlineStr">
@@ -17505,7 +17505,7 @@
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B450" t="inlineStr">
@@ -17543,7 +17543,7 @@
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
@@ -17581,7 +17581,7 @@
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
@@ -17619,7 +17619,7 @@
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
@@ -17657,7 +17657,7 @@
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
@@ -17695,7 +17695,7 @@
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
@@ -17733,7 +17733,7 @@
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B456" t="inlineStr">
@@ -17771,7 +17771,7 @@
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B457" t="inlineStr">
@@ -17809,7 +17809,7 @@
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B458" t="inlineStr">
@@ -17847,7 +17847,7 @@
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B459" t="inlineStr">
@@ -17885,7 +17885,7 @@
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B460" t="inlineStr">
@@ -17923,7 +17923,7 @@
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B461" t="inlineStr">
@@ -17961,7 +17961,7 @@
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B462" t="inlineStr">
@@ -17999,7 +17999,7 @@
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B463" t="inlineStr">
@@ -18037,7 +18037,7 @@
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B464" t="inlineStr">
@@ -18075,7 +18075,7 @@
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B465" t="inlineStr">
@@ -18113,7 +18113,7 @@
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B466" t="inlineStr">
@@ -18151,7 +18151,7 @@
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B467" t="inlineStr">
@@ -18189,7 +18189,7 @@
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
@@ -18227,7 +18227,7 @@
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
@@ -18265,7 +18265,7 @@
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B470" t="inlineStr">
@@ -18303,7 +18303,7 @@
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B471" t="inlineStr">
@@ -18341,7 +18341,7 @@
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B472" t="inlineStr">
@@ -18379,7 +18379,7 @@
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B473" t="inlineStr">
@@ -18417,7 +18417,7 @@
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B474" t="inlineStr">
@@ -18455,7 +18455,7 @@
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B475" t="inlineStr">
@@ -18493,7 +18493,7 @@
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B476" t="inlineStr">
@@ -18531,7 +18531,7 @@
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B477" t="inlineStr">
@@ -18569,7 +18569,7 @@
     <row r="478">
       <c r="A478" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B478" t="inlineStr">
@@ -18607,7 +18607,7 @@
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B479" t="inlineStr">
@@ -18645,7 +18645,7 @@
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B480" t="inlineStr">
@@ -18683,7 +18683,7 @@
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B481" t="inlineStr">
@@ -18721,7 +18721,7 @@
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B482" t="inlineStr">
@@ -18759,7 +18759,7 @@
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B483" t="inlineStr">
@@ -18797,7 +18797,7 @@
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
@@ -18835,7 +18835,7 @@
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B485" t="inlineStr">
@@ -18873,7 +18873,7 @@
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
@@ -18911,7 +18911,7 @@
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
@@ -18949,7 +18949,7 @@
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Ramlager</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
@@ -18987,7 +18987,7 @@
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B489" t="inlineStr">
@@ -19025,7 +19025,7 @@
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>Motorlager</t>
+          <t>Vevlager</t>
         </is>
       </c>
       <c r="B490" t="inlineStr">

</xml_diff>